<commit_message>
creación columnas: 'asignaturas_reprobadas' y 'repitencia'
</commit_message>
<xml_diff>
--- a/investigaciones/teoria mediaombiental de bronfenbrenner y machine learning/estudiantes.xlsx
+++ b/investigaciones/teoria mediaombiental de bronfenbrenner y machine learning/estudiantes.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="25726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="25831"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Danko\Dropbox\00 Doctorado\Paper\Teoria mediaombiental de Bronfenbenner y Machine Learning\estudio\Nueva carpeta\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Danko\Dropbox\00 Programacion\00_portafolio\investigaciones\teoria mediaombiental de bronfenbrenner y machine learning\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7F4E3B0-8D9E-44FD-B2D3-56D2DEDF38A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E770CA42-A422-443D-A896-B7E87A1735FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,21 +16,11 @@
     <sheet name="passengers" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4608" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4610" uniqueCount="197">
   <si>
     <t>genero</t>
   </si>
@@ -616,6 +606,12 @@
   <si>
     <t>vive_con_madre</t>
   </si>
+  <si>
+    <t>asignaturas_reprobadas</t>
+  </si>
+  <si>
+    <t>repitencia_pasada</t>
+  </si>
 </sst>
 </file>
 
@@ -679,28 +675,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -1034,7 +1009,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:DL175"/>
+  <dimension ref="A1:DN175"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" customWidth="1"/>
@@ -1046,9 +1021,10 @@
     <col min="24" max="24" width="19" style="5" customWidth="1"/>
     <col min="25" max="106" width="9.140625" customWidth="1"/>
     <col min="107" max="116" width="3.7109375" customWidth="1"/>
+    <col min="117" max="117" width="4.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1140,7 +1116,7 @@
         <v>25</v>
       </c>
       <c r="AE1" s="1" t="s">
-        <v>26</v>
+        <v>196</v>
       </c>
       <c r="AF1" s="1" t="s">
         <v>27</v>
@@ -1397,8 +1373,14 @@
       <c r="DL1" s="1" t="s">
         <v>183</v>
       </c>
+      <c r="DM1" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="DN1" s="1" t="s">
+        <v>26</v>
+      </c>
     </row>
-    <row r="2" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>102</v>
       </c>
@@ -1744,8 +1726,16 @@
       <c r="DL2" s="2">
         <v>4.7</v>
       </c>
+      <c r="DM2">
+        <f>COUNTIF(DC2:DK2,"&lt;4")</f>
+        <v>2</v>
+      </c>
+      <c r="DN2">
+        <f xml:space="preserve"> IF(OR(AND(DM2=0,DL2&lt;4),AND(DM2=1,DL2&lt;4.5),AND(DM2=2,DL2&lt;5),DM2&gt;=3),1,0)</f>
+        <v>1</v>
+      </c>
     </row>
-    <row r="3" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>103</v>
       </c>
@@ -2091,8 +2081,16 @@
       <c r="DL3" s="2">
         <v>6.7</v>
       </c>
+      <c r="DM3">
+        <f t="shared" ref="DM3:DM66" si="0">COUNTIF(DC3:DK3,"&lt;4")</f>
+        <v>0</v>
+      </c>
+      <c r="DN3">
+        <f t="shared" ref="DN3:DN66" si="1" xml:space="preserve"> IF(OR(AND(DM3=0,DL3&lt;4),AND(DM3=1,DL3&lt;4.5),AND(DM3=2,DL3&lt;5),DM3&gt;=3),1,0)</f>
+        <v>0</v>
+      </c>
     </row>
-    <row r="4" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>102</v>
       </c>
@@ -2438,8 +2436,16 @@
       <c r="DL4" s="2">
         <v>4.9000000000000004</v>
       </c>
+      <c r="DM4">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="DN4">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
     </row>
-    <row r="5" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>102</v>
       </c>
@@ -2785,8 +2791,16 @@
       <c r="DL5" s="2">
         <v>6</v>
       </c>
+      <c r="DM5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="DN5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="6" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>102</v>
       </c>
@@ -3132,8 +3146,16 @@
       <c r="DL6" s="2">
         <v>6</v>
       </c>
+      <c r="DM6">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="DN6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="7" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>103</v>
       </c>
@@ -3479,8 +3501,16 @@
       <c r="DL7" s="2">
         <v>5.9</v>
       </c>
+      <c r="DM7">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="DN7">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="8" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>102</v>
       </c>
@@ -3826,8 +3856,16 @@
       <c r="DL8" s="2">
         <v>5.9</v>
       </c>
+      <c r="DM8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="DN8">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="9" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>102</v>
       </c>
@@ -4173,8 +4211,16 @@
       <c r="DL9" s="2">
         <v>5.4</v>
       </c>
+      <c r="DM9">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="DN9">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="10" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>102</v>
       </c>
@@ -4520,8 +4566,16 @@
       <c r="DL10" s="2">
         <v>6.2</v>
       </c>
+      <c r="DM10">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="DN10">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="11" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>102</v>
       </c>
@@ -4867,8 +4921,16 @@
       <c r="DL11" s="2">
         <v>5.6</v>
       </c>
+      <c r="DM11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="DN11">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="12" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>103</v>
       </c>
@@ -5214,8 +5276,16 @@
       <c r="DL12" s="2">
         <v>5.2</v>
       </c>
+      <c r="DM12">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="DN12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="13" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>103</v>
       </c>
@@ -5561,8 +5631,16 @@
       <c r="DL13" s="2">
         <v>6.2</v>
       </c>
+      <c r="DM13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="DN13">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="14" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>103</v>
       </c>
@@ -5908,8 +5986,16 @@
       <c r="DL14" s="2">
         <v>6.4</v>
       </c>
+      <c r="DM14">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="DN14">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="15" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>102</v>
       </c>
@@ -6255,8 +6341,16 @@
       <c r="DL15" s="2">
         <v>5.6</v>
       </c>
+      <c r="DM15">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="DN15">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="16" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>103</v>
       </c>
@@ -6602,8 +6696,16 @@
       <c r="DL16" s="2">
         <v>5.0999999999999996</v>
       </c>
+      <c r="DM16">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="DN16">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="17" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>103</v>
       </c>
@@ -6949,8 +7051,16 @@
       <c r="DL17" s="2">
         <v>4.2</v>
       </c>
+      <c r="DM17">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="DN17">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
     </row>
-    <row r="18" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>103</v>
       </c>
@@ -7296,8 +7406,16 @@
       <c r="DL18" s="2">
         <v>6.9</v>
       </c>
+      <c r="DM18">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="DN18">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="19" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>102</v>
       </c>
@@ -7643,8 +7761,16 @@
       <c r="DL19" s="2">
         <v>4.5999999999999996</v>
       </c>
+      <c r="DM19">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="DN19">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
     </row>
-    <row r="20" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>103</v>
       </c>
@@ -7990,8 +8116,16 @@
       <c r="DL20" s="2">
         <v>6.1</v>
       </c>
+      <c r="DM20">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="DN20">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="21" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>103</v>
       </c>
@@ -8337,8 +8471,16 @@
       <c r="DL21" s="2">
         <v>5</v>
       </c>
+      <c r="DM21">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="DN21">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="22" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>102</v>
       </c>
@@ -8684,8 +8826,16 @@
       <c r="DL22" s="2">
         <v>6.1</v>
       </c>
+      <c r="DM22">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="DN22">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="23" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>102</v>
       </c>
@@ -9031,8 +9181,16 @@
       <c r="DL23" s="2">
         <v>5.5</v>
       </c>
+      <c r="DM23">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="DN23">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="24" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>103</v>
       </c>
@@ -9378,8 +9536,16 @@
       <c r="DL24" s="2">
         <v>6.3</v>
       </c>
+      <c r="DM24">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="DN24">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="25" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>102</v>
       </c>
@@ -9725,8 +9891,16 @@
       <c r="DL25" s="2">
         <v>6.5</v>
       </c>
+      <c r="DM25">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="DN25">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="26" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>103</v>
       </c>
@@ -10072,8 +10246,16 @@
       <c r="DL26" s="2">
         <v>6.2</v>
       </c>
+      <c r="DM26">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="DN26">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="27" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>101</v>
       </c>
@@ -10419,8 +10601,16 @@
       <c r="DL27" s="2">
         <v>6.4</v>
       </c>
+      <c r="DM27">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="DN27">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="28" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>102</v>
       </c>
@@ -10766,8 +10956,16 @@
       <c r="DL28" s="2">
         <v>4.7</v>
       </c>
+      <c r="DM28">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="DN28">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
     </row>
-    <row r="29" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>103</v>
       </c>
@@ -11113,8 +11311,16 @@
       <c r="DL29" s="2">
         <v>6.7</v>
       </c>
+      <c r="DM29">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="DN29">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="30" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>102</v>
       </c>
@@ -11460,8 +11666,16 @@
       <c r="DL30" s="2">
         <v>5.8</v>
       </c>
+      <c r="DM30">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="DN30">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="31" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>102</v>
       </c>
@@ -11807,8 +12021,16 @@
       <c r="DL31" s="2">
         <v>5.6</v>
       </c>
+      <c r="DM31">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="DN31">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="32" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>103</v>
       </c>
@@ -12154,8 +12376,16 @@
       <c r="DL32" s="2">
         <v>4.4000000000000004</v>
       </c>
+      <c r="DM32">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="DN32">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
     </row>
-    <row r="33" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>103</v>
       </c>
@@ -12501,8 +12731,16 @@
       <c r="DL33" s="2">
         <v>4.5999999999999996</v>
       </c>
+      <c r="DM33">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="DN33">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
     </row>
-    <row r="34" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>103</v>
       </c>
@@ -12848,8 +13086,16 @@
       <c r="DL34" s="2">
         <v>4.8</v>
       </c>
+      <c r="DM34">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="DN34">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
     </row>
-    <row r="35" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>102</v>
       </c>
@@ -13195,8 +13441,16 @@
       <c r="DL35" s="2">
         <v>3.7</v>
       </c>
+      <c r="DM35">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="DN35">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
     </row>
-    <row r="36" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>102</v>
       </c>
@@ -13542,8 +13796,16 @@
       <c r="DL36" s="2">
         <v>5.6</v>
       </c>
+      <c r="DM36">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="DN36">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="37" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>103</v>
       </c>
@@ -13889,8 +14151,16 @@
       <c r="DL37" s="2">
         <v>6.3</v>
       </c>
+      <c r="DM37">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="DN37">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="38" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>103</v>
       </c>
@@ -14236,8 +14506,16 @@
       <c r="DL38" s="2">
         <v>5.9</v>
       </c>
+      <c r="DM38">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="DN38">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="39" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>103</v>
       </c>
@@ -14583,8 +14861,16 @@
       <c r="DL39" s="2">
         <v>5.7</v>
       </c>
+      <c r="DM39">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="DN39">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="40" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>102</v>
       </c>
@@ -14930,8 +15216,16 @@
       <c r="DL40" s="2">
         <v>5.5</v>
       </c>
+      <c r="DM40">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="DN40">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="41" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>103</v>
       </c>
@@ -15277,8 +15571,16 @@
       <c r="DL41" s="2">
         <v>5.6</v>
       </c>
+      <c r="DM41">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="DN41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="42" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>103</v>
       </c>
@@ -15624,8 +15926,16 @@
       <c r="DL42" s="2">
         <v>5</v>
       </c>
+      <c r="DM42">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="DN42">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="43" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>102</v>
       </c>
@@ -15971,8 +16281,16 @@
       <c r="DL43" s="2">
         <v>6</v>
       </c>
+      <c r="DM43">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="DN43">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="44" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>103</v>
       </c>
@@ -16318,8 +16636,16 @@
       <c r="DL44" s="2">
         <v>5.9</v>
       </c>
+      <c r="DM44">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="DN44">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="45" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>103</v>
       </c>
@@ -16665,8 +16991,16 @@
       <c r="DL45" s="2">
         <v>5.6</v>
       </c>
+      <c r="DM45">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="DN45">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="46" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>102</v>
       </c>
@@ -17012,8 +17346,16 @@
       <c r="DL46" s="2">
         <v>5</v>
       </c>
+      <c r="DM46">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="DN46">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="47" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>102</v>
       </c>
@@ -17359,8 +17701,16 @@
       <c r="DL47" s="2">
         <v>4.7</v>
       </c>
+      <c r="DM47">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="DN47">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
     </row>
-    <row r="48" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>102</v>
       </c>
@@ -17706,8 +18056,16 @@
       <c r="DL48" s="2">
         <v>5.7</v>
       </c>
+      <c r="DM48">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="DN48">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="49" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>103</v>
       </c>
@@ -18053,8 +18411,16 @@
       <c r="DL49" s="2">
         <v>4.9000000000000004</v>
       </c>
+      <c r="DM49">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="DN49">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="50" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>102</v>
       </c>
@@ -18400,8 +18766,16 @@
       <c r="DL50" s="2">
         <v>3.8</v>
       </c>
+      <c r="DM50">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="DN50">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
     </row>
-    <row r="51" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>102</v>
       </c>
@@ -18747,8 +19121,16 @@
       <c r="DL51" s="2">
         <v>4.5999999999999996</v>
       </c>
+      <c r="DM51">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="DN51">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
     </row>
-    <row r="52" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>102</v>
       </c>
@@ -19094,8 +19476,16 @@
       <c r="DL52" s="2">
         <v>5.3</v>
       </c>
+      <c r="DM52">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="DN52">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="53" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>103</v>
       </c>
@@ -19441,8 +19831,16 @@
       <c r="DL53" s="2">
         <v>5.8</v>
       </c>
+      <c r="DM53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="DN53">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="54" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>103</v>
       </c>
@@ -19788,8 +20186,16 @@
       <c r="DL54" s="2">
         <v>5.8</v>
       </c>
+      <c r="DM54">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="DN54">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="55" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>103</v>
       </c>
@@ -20135,8 +20541,16 @@
       <c r="DL55" s="2">
         <v>6.3</v>
       </c>
+      <c r="DM55">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="DN55">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="56" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>103</v>
       </c>
@@ -20482,8 +20896,16 @@
       <c r="DL56" s="2">
         <v>5.6</v>
       </c>
+      <c r="DM56">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="DN56">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="57" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>102</v>
       </c>
@@ -20829,8 +21251,16 @@
       <c r="DL57" s="2">
         <v>5.4</v>
       </c>
+      <c r="DM57">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="DN57">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="58" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>103</v>
       </c>
@@ -21176,8 +21606,16 @@
       <c r="DL58" s="2">
         <v>6.2</v>
       </c>
+      <c r="DM58">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="DN58">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="59" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>102</v>
       </c>
@@ -21523,8 +21961,16 @@
       <c r="DL59" s="2">
         <v>5.7</v>
       </c>
+      <c r="DM59">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="DN59">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="60" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>103</v>
       </c>
@@ -21870,8 +22316,16 @@
       <c r="DL60" s="2">
         <v>5.2</v>
       </c>
+      <c r="DM60">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="DN60">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="61" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>104</v>
       </c>
@@ -22217,8 +22671,16 @@
       <c r="DL61" s="2">
         <v>5.5</v>
       </c>
+      <c r="DM61">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="DN61">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="62" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>103</v>
       </c>
@@ -22564,8 +23026,16 @@
       <c r="DL62" s="2">
         <v>6.2</v>
       </c>
+      <c r="DM62">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="DN62">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="63" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>102</v>
       </c>
@@ -22911,8 +23381,16 @@
       <c r="DL63" s="2">
         <v>5.6</v>
       </c>
+      <c r="DM63">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="DN63">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="64" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>102</v>
       </c>
@@ -23258,8 +23736,16 @@
       <c r="DL64" s="2">
         <v>6.7</v>
       </c>
+      <c r="DM64">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="DN64">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="65" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>102</v>
       </c>
@@ -23605,8 +24091,16 @@
       <c r="DL65" s="2">
         <v>6.2</v>
       </c>
+      <c r="DM65">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="DN65">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="66" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>103</v>
       </c>
@@ -23952,8 +24446,16 @@
       <c r="DL66" s="2">
         <v>5.9</v>
       </c>
+      <c r="DM66">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="DN66">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="67" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>103</v>
       </c>
@@ -24299,8 +24801,16 @@
       <c r="DL67" s="2">
         <v>5.0999999999999996</v>
       </c>
+      <c r="DM67">
+        <f t="shared" ref="DM67:DM130" si="2">COUNTIF(DC67:DK67,"&lt;4")</f>
+        <v>2</v>
+      </c>
+      <c r="DN67">
+        <f t="shared" ref="DN67:DN130" si="3" xml:space="preserve"> IF(OR(AND(DM67=0,DL67&lt;4),AND(DM67=1,DL67&lt;4.5),AND(DM67=2,DL67&lt;5),DM67&gt;=3),1,0)</f>
+        <v>0</v>
+      </c>
     </row>
-    <row r="68" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>103</v>
       </c>
@@ -24646,8 +25156,16 @@
       <c r="DL68" s="2">
         <v>6.2</v>
       </c>
+      <c r="DM68">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DN68">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="69" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>102</v>
       </c>
@@ -24993,8 +25511,16 @@
       <c r="DL69" s="2">
         <v>4.5999999999999996</v>
       </c>
+      <c r="DM69">
+        <f t="shared" si="2"/>
+        <v>2</v>
+      </c>
+      <c r="DN69">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
     </row>
-    <row r="70" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>103</v>
       </c>
@@ -25340,8 +25866,16 @@
       <c r="DL70" s="2">
         <v>6.2</v>
       </c>
+      <c r="DM70">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DN70">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="71" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>103</v>
       </c>
@@ -25687,8 +26221,16 @@
       <c r="DL71" s="2">
         <v>5.7</v>
       </c>
+      <c r="DM71">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DN71">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="72" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>103</v>
       </c>
@@ -26034,8 +26576,16 @@
       <c r="DL72" s="2">
         <v>6.1</v>
       </c>
+      <c r="DM72">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DN72">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="73" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>102</v>
       </c>
@@ -26381,8 +26931,16 @@
       <c r="DL73" s="2">
         <v>5.5</v>
       </c>
+      <c r="DM73">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DN73">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="74" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>103</v>
       </c>
@@ -26728,8 +27286,16 @@
       <c r="DL74" s="2">
         <v>6.1</v>
       </c>
+      <c r="DM74">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DN74">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="75" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>102</v>
       </c>
@@ -27075,8 +27641,16 @@
       <c r="DL75" s="2">
         <v>6.7</v>
       </c>
+      <c r="DM75">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DN75">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="76" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>102</v>
       </c>
@@ -27422,8 +27996,16 @@
       <c r="DL76" s="2">
         <v>6.6</v>
       </c>
+      <c r="DM76">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DN76">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="77" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>102</v>
       </c>
@@ -27769,8 +28351,16 @@
       <c r="DL77" s="2">
         <v>6.7</v>
       </c>
+      <c r="DM77">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DN77">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="78" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>103</v>
       </c>
@@ -28116,8 +28706,16 @@
       <c r="DL78" s="2">
         <v>6.2</v>
       </c>
+      <c r="DM78">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DN78">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="79" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>102</v>
       </c>
@@ -28463,8 +29061,16 @@
       <c r="DL79" s="2">
         <v>6</v>
       </c>
+      <c r="DM79">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DN79">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="80" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>105</v>
       </c>
@@ -28810,8 +29416,16 @@
       <c r="DL80" s="2">
         <v>6.1</v>
       </c>
+      <c r="DM80">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DN80">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="81" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>102</v>
       </c>
@@ -29157,8 +29771,16 @@
       <c r="DL81" s="2">
         <v>6.3</v>
       </c>
+      <c r="DM81">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DN81">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="82" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>102</v>
       </c>
@@ -29504,8 +30126,16 @@
       <c r="DL82" s="2">
         <v>5.5</v>
       </c>
+      <c r="DM82">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="DN82">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="83" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>102</v>
       </c>
@@ -29851,8 +30481,16 @@
       <c r="DL83" s="2">
         <v>6.2</v>
       </c>
+      <c r="DM83">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DN83">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="84" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>103</v>
       </c>
@@ -30198,8 +30836,16 @@
       <c r="DL84" s="2">
         <v>5.7</v>
       </c>
+      <c r="DM84">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DN84">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="85" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>103</v>
       </c>
@@ -30545,8 +31191,16 @@
       <c r="DL85" s="2">
         <v>5.5</v>
       </c>
+      <c r="DM85">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DN85">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="86" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>102</v>
       </c>
@@ -30892,8 +31546,16 @@
       <c r="DL86" s="2">
         <v>6.6</v>
       </c>
+      <c r="DM86">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DN86">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="87" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>103</v>
       </c>
@@ -31239,8 +31901,16 @@
       <c r="DL87" s="2">
         <v>5.8</v>
       </c>
+      <c r="DM87">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DN87">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="88" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>102</v>
       </c>
@@ -31586,8 +32256,16 @@
       <c r="DL88" s="2">
         <v>5.8</v>
       </c>
+      <c r="DM88">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DN88">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="89" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>103</v>
       </c>
@@ -31933,8 +32611,16 @@
       <c r="DL89" s="2">
         <v>6.1</v>
       </c>
+      <c r="DM89">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DN89">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="90" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>102</v>
       </c>
@@ -32280,8 +32966,16 @@
       <c r="DL90" s="2">
         <v>6.7</v>
       </c>
+      <c r="DM90">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DN90">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="91" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>102</v>
       </c>
@@ -32627,8 +33321,16 @@
       <c r="DL91" s="2">
         <v>5.0999999999999996</v>
       </c>
+      <c r="DM91">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DN91">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="92" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>103</v>
       </c>
@@ -32974,8 +33676,16 @@
       <c r="DL92" s="2">
         <v>5.8</v>
       </c>
+      <c r="DM92">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DN92">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="93" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>103</v>
       </c>
@@ -33321,8 +34031,16 @@
       <c r="DL93" s="2">
         <v>5.6</v>
       </c>
+      <c r="DM93">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DN93">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="94" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>102</v>
       </c>
@@ -33668,8 +34386,16 @@
       <c r="DL94" s="2">
         <v>6.6</v>
       </c>
+      <c r="DM94">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DN94">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="95" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>102</v>
       </c>
@@ -34015,8 +34741,16 @@
       <c r="DL95" s="2">
         <v>5.9</v>
       </c>
+      <c r="DM95">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DN95">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="96" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>103</v>
       </c>
@@ -34362,8 +35096,16 @@
       <c r="DL96" s="2">
         <v>5.6</v>
       </c>
+      <c r="DM96">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DN96">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="97" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>103</v>
       </c>
@@ -34709,8 +35451,16 @@
       <c r="DL97" s="2">
         <v>5.8</v>
       </c>
+      <c r="DM97">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DN97">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="98" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>106</v>
       </c>
@@ -35056,8 +35806,16 @@
       <c r="DL98" s="2">
         <v>5.5</v>
       </c>
+      <c r="DM98">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DN98">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="99" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>103</v>
       </c>
@@ -35403,8 +36161,16 @@
       <c r="DL99" s="2">
         <v>4.8</v>
       </c>
+      <c r="DM99">
+        <f t="shared" si="2"/>
+        <v>3</v>
+      </c>
+      <c r="DN99">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
     </row>
-    <row r="100" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>103</v>
       </c>
@@ -35750,8 +36516,16 @@
       <c r="DL100" s="2">
         <v>6.3</v>
       </c>
+      <c r="DM100">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DN100">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="101" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>103</v>
       </c>
@@ -36097,8 +36871,16 @@
       <c r="DL101" s="2">
         <v>4.7</v>
       </c>
+      <c r="DM101">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="DN101">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="102" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>102</v>
       </c>
@@ -36444,8 +37226,16 @@
       <c r="DL102" s="2">
         <v>5</v>
       </c>
+      <c r="DM102">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="DN102">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="103" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>103</v>
       </c>
@@ -36791,8 +37581,16 @@
       <c r="DL103" s="2">
         <v>4.7</v>
       </c>
+      <c r="DM103">
+        <f t="shared" si="2"/>
+        <v>2</v>
+      </c>
+      <c r="DN103">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
     </row>
-    <row r="104" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>102</v>
       </c>
@@ -37138,8 +37936,16 @@
       <c r="DL104" s="2">
         <v>5.6</v>
       </c>
+      <c r="DM104">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DN104">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="105" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>102</v>
       </c>
@@ -37485,8 +38291,16 @@
       <c r="DL105" s="2">
         <v>6.7</v>
       </c>
+      <c r="DM105">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DN105">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="106" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>103</v>
       </c>
@@ -37832,8 +38646,16 @@
       <c r="DL106" s="2">
         <v>5.4</v>
       </c>
+      <c r="DM106">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DN106">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="107" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>102</v>
       </c>
@@ -38179,8 +39001,16 @@
       <c r="DL107" s="2">
         <v>4.9000000000000004</v>
       </c>
+      <c r="DM107">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="DN107">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="108" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>102</v>
       </c>
@@ -38526,8 +39356,16 @@
       <c r="DL108" s="2">
         <v>5</v>
       </c>
+      <c r="DM108">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DN108">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="109" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>102</v>
       </c>
@@ -38873,8 +39711,16 @@
       <c r="DL109" s="2">
         <v>5.5</v>
       </c>
+      <c r="DM109">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DN109">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="110" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>103</v>
       </c>
@@ -39220,8 +40066,16 @@
       <c r="DL110" s="2">
         <v>6.3</v>
       </c>
+      <c r="DM110">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DN110">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="111" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>105</v>
       </c>
@@ -39567,8 +40421,16 @@
       <c r="DL111" s="2">
         <v>6.1</v>
       </c>
+      <c r="DM111">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DN111">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="112" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>106</v>
       </c>
@@ -39914,8 +40776,16 @@
       <c r="DL112" s="2">
         <v>5.2</v>
       </c>
+      <c r="DM112">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="DN112">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="113" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>103</v>
       </c>
@@ -40261,8 +41131,16 @@
       <c r="DL113" s="2">
         <v>4.5999999999999996</v>
       </c>
+      <c r="DM113">
+        <f t="shared" si="2"/>
+        <v>4</v>
+      </c>
+      <c r="DN113">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
     </row>
-    <row r="114" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>103</v>
       </c>
@@ -40608,8 +41486,16 @@
       <c r="DL114" s="2">
         <v>6.8</v>
       </c>
+      <c r="DM114">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DN114">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="115" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>102</v>
       </c>
@@ -40955,8 +41841,16 @@
       <c r="DL115" s="2">
         <v>5.3</v>
       </c>
+      <c r="DM115">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="DN115">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="116" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>103</v>
       </c>
@@ -41302,8 +42196,16 @@
       <c r="DL116" s="2">
         <v>6.7</v>
       </c>
+      <c r="DM116">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DN116">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="117" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>105</v>
       </c>
@@ -41649,8 +42551,16 @@
       <c r="DL117" s="2">
         <v>4.9000000000000004</v>
       </c>
+      <c r="DM117">
+        <f t="shared" si="2"/>
+        <v>2</v>
+      </c>
+      <c r="DN117">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
     </row>
-    <row r="118" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>103</v>
       </c>
@@ -41996,8 +42906,16 @@
       <c r="DL118" s="2">
         <v>5.3</v>
       </c>
+      <c r="DM118">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="DN118">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="119" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>105</v>
       </c>
@@ -42343,8 +43261,16 @@
       <c r="DL119" s="2">
         <v>6.1</v>
       </c>
+      <c r="DM119">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DN119">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="120" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>103</v>
       </c>
@@ -42690,8 +43616,16 @@
       <c r="DL120" s="2">
         <v>6.7</v>
       </c>
+      <c r="DM120">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DN120">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="121" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>103</v>
       </c>
@@ -43037,8 +43971,16 @@
       <c r="DL121" s="2">
         <v>4.8</v>
       </c>
+      <c r="DM121">
+        <f t="shared" si="2"/>
+        <v>2</v>
+      </c>
+      <c r="DN121">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
     </row>
-    <row r="122" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>103</v>
       </c>
@@ -43384,8 +44326,16 @@
       <c r="DL122" s="2">
         <v>4.8</v>
       </c>
+      <c r="DM122">
+        <f t="shared" si="2"/>
+        <v>2</v>
+      </c>
+      <c r="DN122">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
     </row>
-    <row r="123" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>102</v>
       </c>
@@ -43731,8 +44681,16 @@
       <c r="DL123" s="2">
         <v>6.9</v>
       </c>
+      <c r="DM123">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DN123">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="124" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>102</v>
       </c>
@@ -44078,8 +45036,16 @@
       <c r="DL124" s="2">
         <v>4.9000000000000004</v>
       </c>
+      <c r="DM124">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="DN124">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="125" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>103</v>
       </c>
@@ -44425,8 +45391,16 @@
       <c r="DL125" s="2">
         <v>6.1</v>
       </c>
+      <c r="DM125">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DN125">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="126" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>103</v>
       </c>
@@ -44772,8 +45746,16 @@
       <c r="DL126" s="2">
         <v>6.8</v>
       </c>
+      <c r="DM126">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DN126">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="127" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>102</v>
       </c>
@@ -45119,8 +46101,16 @@
       <c r="DL127" s="2">
         <v>5.4</v>
       </c>
+      <c r="DM127">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="DN127">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="128" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>102</v>
       </c>
@@ -45466,8 +46456,16 @@
       <c r="DL128" s="2">
         <v>5.7</v>
       </c>
+      <c r="DM128">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="DN128">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="129" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>103</v>
       </c>
@@ -45813,8 +46811,16 @@
       <c r="DL129" s="2">
         <v>4.9000000000000004</v>
       </c>
+      <c r="DM129">
+        <f t="shared" si="2"/>
+        <v>2</v>
+      </c>
+      <c r="DN129">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
     </row>
-    <row r="130" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>103</v>
       </c>
@@ -46160,8 +47166,16 @@
       <c r="DL130" s="2">
         <v>5.5</v>
       </c>
+      <c r="DM130">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DN130">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="131" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>102</v>
       </c>
@@ -46507,8 +47521,16 @@
       <c r="DL131" s="2">
         <v>5.6</v>
       </c>
+      <c r="DM131">
+        <f t="shared" ref="DM131:DM175" si="4">COUNTIF(DC131:DK131,"&lt;4")</f>
+        <v>0</v>
+      </c>
+      <c r="DN131">
+        <f t="shared" ref="DN131:DN175" si="5" xml:space="preserve"> IF(OR(AND(DM131=0,DL131&lt;4),AND(DM131=1,DL131&lt;4.5),AND(DM131=2,DL131&lt;5),DM131&gt;=3),1,0)</f>
+        <v>0</v>
+      </c>
     </row>
-    <row r="132" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>102</v>
       </c>
@@ -46854,8 +47876,16 @@
       <c r="DL132" s="2">
         <v>6.3</v>
       </c>
+      <c r="DM132">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DN132">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="133" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>103</v>
       </c>
@@ -47201,8 +48231,16 @@
       <c r="DL133" s="2">
         <v>5.2</v>
       </c>
+      <c r="DM133">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="DN133">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="134" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>102</v>
       </c>
@@ -47548,8 +48586,16 @@
       <c r="DL134" s="2">
         <v>5.8</v>
       </c>
+      <c r="DM134">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DN134">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="135" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>103</v>
       </c>
@@ -47895,8 +48941,16 @@
       <c r="DL135" s="2">
         <v>6.1</v>
       </c>
+      <c r="DM135">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DN135">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="136" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>102</v>
       </c>
@@ -48242,8 +49296,16 @@
       <c r="DL136" s="2">
         <v>6.2</v>
       </c>
+      <c r="DM136">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DN136">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="137" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>103</v>
       </c>
@@ -48589,8 +49651,16 @@
       <c r="DL137" s="2">
         <v>5.4</v>
       </c>
+      <c r="DM137">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="DN137">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="138" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>102</v>
       </c>
@@ -48936,8 +50006,16 @@
       <c r="DL138" s="2">
         <v>6.1</v>
       </c>
+      <c r="DM138">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DN138">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="139" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>102</v>
       </c>
@@ -49283,8 +50361,16 @@
       <c r="DL139" s="2">
         <v>5.5</v>
       </c>
+      <c r="DM139">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DN139">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="140" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>103</v>
       </c>
@@ -49630,8 +50716,16 @@
       <c r="DL140" s="2">
         <v>4.9000000000000004</v>
       </c>
+      <c r="DM140">
+        <f t="shared" si="4"/>
+        <v>2</v>
+      </c>
+      <c r="DN140">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
     </row>
-    <row r="141" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>103</v>
       </c>
@@ -49977,8 +51071,16 @@
       <c r="DL141" s="2">
         <v>5.7</v>
       </c>
+      <c r="DM141">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DN141">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="142" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>103</v>
       </c>
@@ -50324,8 +51426,16 @@
       <c r="DL142" s="2">
         <v>6.1</v>
       </c>
+      <c r="DM142">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DN142">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="143" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>103</v>
       </c>
@@ -50671,8 +51781,16 @@
       <c r="DL143" s="2">
         <v>5.8</v>
       </c>
+      <c r="DM143">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DN143">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="144" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>102</v>
       </c>
@@ -51018,8 +52136,16 @@
       <c r="DL144" s="2">
         <v>5.4</v>
       </c>
+      <c r="DM144">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="DN144">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="145" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>102</v>
       </c>
@@ -51365,8 +52491,16 @@
       <c r="DL145" s="2">
         <v>5.7</v>
       </c>
+      <c r="DM145">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DN145">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="146" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>103</v>
       </c>
@@ -51712,8 +52846,16 @@
       <c r="DL146" s="2">
         <v>6.6</v>
       </c>
+      <c r="DM146">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DN146">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="147" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>103</v>
       </c>
@@ -52059,8 +53201,16 @@
       <c r="DL147" s="2">
         <v>6.8</v>
       </c>
+      <c r="DM147">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DN147">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="148" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>102</v>
       </c>
@@ -52406,8 +53556,16 @@
       <c r="DL148" s="2">
         <v>7</v>
       </c>
+      <c r="DM148">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DN148">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="149" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>102</v>
       </c>
@@ -52753,8 +53911,16 @@
       <c r="DL149" s="2">
         <v>5.4</v>
       </c>
+      <c r="DM149">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DN149">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="150" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>103</v>
       </c>
@@ -53100,8 +54266,16 @@
       <c r="DL150" s="2">
         <v>5.8</v>
       </c>
+      <c r="DM150">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DN150">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="151" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>103</v>
       </c>
@@ -53447,8 +54621,16 @@
       <c r="DL151" s="2">
         <v>4.9000000000000004</v>
       </c>
+      <c r="DM151">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DN151">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="152" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>103</v>
       </c>
@@ -53794,8 +54976,16 @@
       <c r="DL152" s="2">
         <v>5.4</v>
       </c>
+      <c r="DM152">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DN152">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="153" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>102</v>
       </c>
@@ -54141,8 +55331,16 @@
       <c r="DL153" s="2">
         <v>5.7</v>
       </c>
+      <c r="DM153">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DN153">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="154" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>102</v>
       </c>
@@ -54488,8 +55686,16 @@
       <c r="DL154" s="2">
         <v>6.1</v>
       </c>
+      <c r="DM154">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DN154">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="155" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>103</v>
       </c>
@@ -54835,8 +56041,16 @@
       <c r="DL155" s="2">
         <v>5.5</v>
       </c>
+      <c r="DM155">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DN155">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="156" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
         <v>103</v>
       </c>
@@ -55182,8 +56396,16 @@
       <c r="DL156" s="2">
         <v>5.6</v>
       </c>
+      <c r="DM156">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DN156">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="157" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>103</v>
       </c>
@@ -55529,8 +56751,16 @@
       <c r="DL157" s="2">
         <v>6.4</v>
       </c>
+      <c r="DM157">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DN157">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="158" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
         <v>105</v>
       </c>
@@ -55876,8 +57106,16 @@
       <c r="DL158" s="2">
         <v>5.0999999999999996</v>
       </c>
+      <c r="DM158">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="DN158">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="159" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
         <v>102</v>
       </c>
@@ -56223,8 +57461,16 @@
       <c r="DL159" s="2">
         <v>5.9</v>
       </c>
+      <c r="DM159">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DN159">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="160" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
         <v>103</v>
       </c>
@@ -56570,8 +57816,16 @@
       <c r="DL160" s="2">
         <v>6.3</v>
       </c>
+      <c r="DM160">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DN160">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="161" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>102</v>
       </c>
@@ -56917,8 +58171,16 @@
       <c r="DL161" s="2">
         <v>5.5</v>
       </c>
+      <c r="DM161">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DN161">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="162" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
         <v>103</v>
       </c>
@@ -57264,8 +58526,16 @@
       <c r="DL162" s="2">
         <v>6.8</v>
       </c>
+      <c r="DM162">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DN162">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="163" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
         <v>103</v>
       </c>
@@ -57611,8 +58881,16 @@
       <c r="DL163" s="2">
         <v>6.6</v>
       </c>
+      <c r="DM163">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DN163">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="164" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
         <v>103</v>
       </c>
@@ -57958,8 +59236,16 @@
       <c r="DL164" s="2">
         <v>6.3</v>
       </c>
+      <c r="DM164">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DN164">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="165" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
         <v>102</v>
       </c>
@@ -58305,8 +59591,16 @@
       <c r="DL165" s="2">
         <v>5.2</v>
       </c>
+      <c r="DM165">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DN165">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="166" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
         <v>102</v>
       </c>
@@ -58652,8 +59946,16 @@
       <c r="DL166" s="2">
         <v>5.2</v>
       </c>
+      <c r="DM166">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DN166">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="167" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
         <v>103</v>
       </c>
@@ -58999,8 +60301,16 @@
       <c r="DL167" s="2">
         <v>6</v>
       </c>
+      <c r="DM167">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DN167">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="168" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
         <v>102</v>
       </c>
@@ -59346,8 +60656,16 @@
       <c r="DL168" s="2">
         <v>5.8</v>
       </c>
+      <c r="DM168">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DN168">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="169" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
         <v>102</v>
       </c>
@@ -59693,8 +61011,16 @@
       <c r="DL169" s="2">
         <v>5.8</v>
       </c>
+      <c r="DM169">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DN169">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="170" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
         <v>102</v>
       </c>
@@ -60040,8 +61366,16 @@
       <c r="DL170" s="2">
         <v>6.5</v>
       </c>
+      <c r="DM170">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DN170">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="171" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
         <v>103</v>
       </c>
@@ -60387,8 +61721,16 @@
       <c r="DL171" s="2">
         <v>5.7</v>
       </c>
+      <c r="DM171">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DN171">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="172" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
         <v>102</v>
       </c>
@@ -60734,8 +62076,16 @@
       <c r="DL172" s="2">
         <v>6.1</v>
       </c>
+      <c r="DM172">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DN172">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="173" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
         <v>102</v>
       </c>
@@ -61081,8 +62431,16 @@
       <c r="DL173" s="2">
         <v>6.3</v>
       </c>
+      <c r="DM173">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DN173">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="174" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
         <v>103</v>
       </c>
@@ -61428,8 +62786,16 @@
       <c r="DL174" s="2">
         <v>6.2</v>
       </c>
+      <c r="DM174">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DN174">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="175" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:118" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
         <v>103</v>
       </c>
@@ -61774,6 +63140,14 @@
       </c>
       <c r="DL175" s="2">
         <v>5.6</v>
+      </c>
+      <c r="DM175">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DN175">
+        <f t="shared" si="5"/>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
comparación mediante estadísticos descriptivos entre alumnos repitentes y alumnos promovidos
</commit_message>
<xml_diff>
--- a/investigaciones/teoria mediaombiental de bronfenbrenner y machine learning/estudiantes.xlsx
+++ b/investigaciones/teoria mediaombiental de bronfenbrenner y machine learning/estudiantes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Danko\Dropbox\00 Programacion\00_portafolio\investigaciones\teoria mediaombiental de bronfenbrenner y machine learning\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E770CA42-A422-443D-A896-B7E87A1735FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98ACFDD9-5C6F-499B-92C4-CD48F4D55FF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38663,7 +38663,7 @@
         <v>14</v>
       </c>
       <c r="C107">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="D107">
         <v>1.7</v>

</xml_diff>